<commit_message>
Upated with sending first message and delete it right away
</commit_message>
<xml_diff>
--- a/vehicle_list_8801977158626.xlsx
+++ b/vehicle_list_8801977158626.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,32 +418,18 @@
         <v>Test-1</v>
       </c>
       <c r="B2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
       <c r="D2" t="str">
-        <v>Ashraf-1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Test-2</v>
-      </c>
-      <c r="B3" t="b">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Ashraf-2</v>
+        <v>Buddy 1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>